<commit_message>
Removed fixed noise and got training plots to always decrease.
</commit_message>
<xml_diff>
--- a/data/output/20260922/pureComponents_filled.xlsx
+++ b/data/output/20260922/pureComponents_filled.xlsx
@@ -491,12 +491,12 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>226.3892895068535</v>
+        <v>230.5285601407318</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>8.092697027255742</v>
+        <v>8.218579856978019</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -517,12 +517,12 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>450.3011832115711</v>
+        <v>280.6272773554851</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>-191.4365340526395</v>
+        <v>5.324332267600289</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -543,12 +543,12 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>251.8661107120695</v>
+        <v>258.0220272860158</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>10.53118778433254</v>
+        <v>10.86072117746967</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -569,12 +569,12 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>423.4580742726941</v>
+        <v>289.5485006821258</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>160.2567452866502</v>
+        <v>12.86724069769583</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -595,12 +595,12 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>227.4809965371188</v>
+        <v>217.721040797028</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>10.03470583257606</v>
+        <v>9.201250578834143</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -621,12 +621,12 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>499.9677229649849</v>
+        <v>298.9230725109284</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>-52.91311373437054</v>
+        <v>12.00235307737671</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -647,12 +647,12 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>522.2579954860856</v>
+        <v>620.5705802601036</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>49.39676426026924</v>
+        <v>24.50898429830133</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -673,12 +673,12 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>356.432002110875</v>
+        <v>310.5351298771114</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>19.73137960112631</v>
+        <v>10.53613642935987</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -699,12 +699,12 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>703.434473107194</v>
+        <v>813.4528537523943</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>33.137248280394</v>
+        <v>25.63856825377426</v>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -725,12 +725,12 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>245.7987390237712</v>
+        <v>243.4865039945783</v>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>8.14003638974062</v>
+        <v>8.078937119136503</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -751,12 +751,12 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>389.2439188910884</v>
+        <v>171.831594423355</v>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>79.15850037556592</v>
+        <v>6.708681385557764</v>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -777,12 +777,12 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>385.4352795512679</v>
+        <v>260.614629597831</v>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>42.75012945138688</v>
+        <v>9.147753496969308</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -803,12 +803,12 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>187.2667656788124</v>
+        <v>181.2294101301109</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>6.207543249236824</v>
+        <v>6.00215753929527</v>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -829,12 +829,12 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>234.7663288068059</v>
+        <v>224.4681653878412</v>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>10.91574654358259</v>
+        <v>10.32400807911261</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -855,12 +855,12 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>348.4115254173495</v>
+        <v>119.8921695248892</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>35.96317781896198</v>
+        <v>3.618684123501609</v>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -881,12 +881,12 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>310.1181829155213</v>
+        <v>283.1115522992301</v>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
-        <v>18.83509438849234</v>
+        <v>14.30054841045704</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -907,12 +907,12 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>406.5756940760526</v>
+        <v>147.4891082691907</v>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
-        <v>128.9856813544949</v>
+        <v>5.701811343694116</v>
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -933,12 +933,12 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>319.9699338330606</v>
+        <v>223.1330853050393</v>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
-        <v>18.4333348524455</v>
+        <v>7.084764141270908</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -959,12 +959,12 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>326.4810764010267</v>
+        <v>204.682921829022</v>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
-        <v>25.02976008472713</v>
+        <v>7.547390227858426</v>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -985,12 +985,12 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>158.4976684731346</v>
+        <v>146.0176258382641</v>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>5.207380181768777</v>
+        <v>4.745191002580068</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -1011,12 +1011,12 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>342.2077960428663</v>
+        <v>206.3317690555035</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>35.10419647335656</v>
+        <v>8.810765928619837</v>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -1037,12 +1037,12 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>387.2269891417278</v>
+        <v>219.9356143716117</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
-        <v>63.52825053077514</v>
+        <v>8.904997046417753</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
@@ -1063,12 +1063,12 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>582.9843277030036</v>
+        <v>324.8858149551142</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
-        <v>-19.31319426951159</v>
+        <v>12.29757140675225</v>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
@@ -1089,12 +1089,12 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>918.5868607059249</v>
+        <v>897.3503321782962</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
-        <v>20.65972133376436</v>
+        <v>20.10986367569337</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1115,12 +1115,12 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>381.3172928364659</v>
+        <v>327.8699504493716</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
-        <v>27.14027069905195</v>
+        <v>11.77031869105104</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
@@ -1141,12 +1141,12 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>171.0398804679537</v>
+        <v>175.9936288449216</v>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
-        <v>5.71422486370682</v>
+        <v>5.897597573930398</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -1167,12 +1167,12 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>209.9915721786144</v>
+        <v>186.8977944487656</v>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
-        <v>7.57787209793128</v>
+        <v>6.646747532657145</v>
       </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
@@ -1193,12 +1193,12 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>346.7683839583349</v>
+        <v>159.8358667878036</v>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
-        <v>39.3888421190459</v>
+        <v>6.005338938476806</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
@@ -1219,12 +1219,12 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>197.9081943516057</v>
+        <v>190.7199357722525</v>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
-        <v>6.70523962523245</v>
+        <v>6.404152470348823</v>
       </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
@@ -1245,12 +1245,12 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>349.765465914536</v>
+        <v>271.821000306116</v>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="n">
-        <v>29.32556113545014</v>
+        <v>12.18657463626084</v>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
@@ -1271,12 +1271,12 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>501.7924243507575</v>
+        <v>265.8211763515511</v>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>-63.4674126522944</v>
+        <v>10.74379049118423</v>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
@@ -1297,12 +1297,12 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>991.5371623508091</v>
+        <v>973.4971391132553</v>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>25.37172393918426</v>
+        <v>25.7796215783605</v>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
@@ -1323,12 +1323,12 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>525.1242213110955</v>
+        <v>652.8253975553612</v>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>53.14280116447933</v>
+        <v>24.20512501055465</v>
       </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
@@ -1349,12 +1349,12 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>193.6613801406016</v>
+        <v>178.0462564070317</v>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
-        <v>5.440667333186951</v>
+        <v>5.002051537283394</v>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
@@ -1375,12 +1375,12 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>218.0337498063079</v>
+        <v>210.4835487112126</v>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
-        <v>12.27906347435003</v>
+        <v>11.62954266891588</v>
       </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
@@ -1401,12 +1401,12 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>775.8756503773725</v>
+        <v>836.9657162841271</v>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
-        <v>29.40796543745662</v>
+        <v>25.55801144591133</v>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
@@ -1427,12 +1427,12 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>505.7480549392224</v>
+        <v>314.3849130027971</v>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
-        <v>-42.48405209319603</v>
+        <v>12.36220784399122</v>
       </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
@@ -1453,12 +1453,12 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>920.8646092397905</v>
+        <v>941.3822368859518</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
-        <v>26.68192273838175</v>
+        <v>29.16181180896738</v>
       </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
@@ -1479,12 +1479,12 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>518.6883891234099</v>
+        <v>605.6533090260397</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
-        <v>47.50047023522843</v>
+        <v>23.93689418370924</v>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
@@ -1505,12 +1505,12 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>414.1752514795634</v>
+        <v>400.0698603080006</v>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
-        <v>14.59561515971462</v>
+        <v>14.04336509926725</v>
       </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
@@ -1531,12 +1531,12 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>409.3940432217667</v>
+        <v>369.3261914635831</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
-        <v>24.6081729776041</v>
+        <v>21.38215395923003</v>
       </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
@@ -1557,12 +1557,12 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>469.487295515833</v>
+        <v>408.9187171577294</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
-        <v>11.01407567445179</v>
+        <v>9.661157139776011</v>
       </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
@@ -1583,12 +1583,12 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>446.5707495750706</v>
+        <v>416.030095408967</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
-        <v>16.98422981645019</v>
+        <v>15.53112752357966</v>
       </c>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
@@ -1609,12 +1609,12 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>445.2457014155436</v>
+        <v>445.0421429510677</v>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>28.0399530896236</v>
+        <v>23.16235723016841</v>
       </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
@@ -1635,12 +1635,12 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>524.8662166871308</v>
+        <v>519.1051742680455</v>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
-        <v>16.74382374937468</v>
+        <v>16.80093378793335</v>
       </c>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
@@ -1661,12 +1661,12 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>497.8406231404214</v>
+        <v>517.7394884356055</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
-        <v>48.20352735502853</v>
+        <v>50.49074828756897</v>
       </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
@@ -1687,12 +1687,12 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>465.2481638931996</v>
+        <v>463.344199893606</v>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
-        <v>27.60975355685752</v>
+        <v>20.2264858518564</v>
       </c>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
@@ -1713,12 +1713,12 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>528.3450591688693</v>
+        <v>528.0177733738508</v>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="n">
-        <v>26.94180774226215</v>
+        <v>26.07672395943744</v>
       </c>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>408.7690753608349</v>
+        <v>413.2245276675304</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
-        <v>17.67838115849661</v>
+        <v>21.63457587142056</v>
       </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
@@ -1765,12 +1765,12 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>370.8687945277871</v>
+        <v>358.0023127067872</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
-        <v>13.92327352169858</v>
+        <v>13.61056997989314</v>
       </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
@@ -1791,12 +1791,12 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>469.6567218693743</v>
+        <v>477.1484229395755</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
-        <v>29.39428131939636</v>
+        <v>20.89166744696251</v>
       </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
@@ -1817,12 +1817,12 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>665.9568476071037</v>
+        <v>618.0666352710888</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
-        <v>21.71347510611127</v>
+        <v>20.3305892935719</v>
       </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
@@ -1843,12 +1843,12 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>460.055267910623</v>
+        <v>467.7463813675583</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
-        <v>36.01194381785113</v>
+        <v>21.55256924431178</v>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
@@ -1869,12 +1869,12 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>595.7530177906182</v>
+        <v>621.8777712385762</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>33.00591659125514</v>
+        <v>35.72453721443676</v>
       </c>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
@@ -1895,12 +1895,12 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>380.0230060656417</v>
+        <v>392.4227631630488</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
-        <v>40.66645921771299</v>
+        <v>41.37381407968098</v>
       </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
@@ -1921,12 +1921,12 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>698.3088112934618</v>
+        <v>301.6057056798974</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
-        <v>3.321720839474093</v>
+        <v>1.509591229103531</v>
       </c>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
@@ -1947,12 +1947,12 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>402.0641178859806</v>
+        <v>415.892844833454</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="n">
-        <v>38.19918785447543</v>
+        <v>39.29695603483751</v>
       </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
@@ -1973,12 +1973,12 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>595.1090445991102</v>
+        <v>530.3995707222064</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="n">
-        <v>7.685670527933858</v>
+        <v>7.17385580142242</v>
       </c>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
@@ -1999,12 +1999,12 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>445.682160448657</v>
+        <v>471.5072030269084</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="n">
-        <v>62.34772317260103</v>
+        <v>65.98825674812392</v>
       </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
@@ -2025,12 +2025,12 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>467.04608389043</v>
+        <v>445.732298841306</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="n">
-        <v>18.6784586277804</v>
+        <v>16.30911515392334</v>
       </c>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr"/>
@@ -2051,12 +2051,12 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>159.9355861003573</v>
+        <v>157.8551200934199</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="n">
-        <v>6.81494083153923</v>
+        <v>6.685480711033231</v>
       </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
@@ -2077,12 +2077,12 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>714.6626690710948</v>
+        <v>647.3257466924889</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="n">
-        <v>8.928829899198931</v>
+        <v>7.688863518536179</v>
       </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
@@ -2103,12 +2103,12 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>297.390542360336</v>
+        <v>329.4695477701716</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="n">
-        <v>11.14460220566998</v>
+        <v>14.4621613489244</v>
       </c>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
@@ -2129,12 +2129,12 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>156.3528385658726</v>
+        <v>285.9194523508135</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="n">
-        <v>3.641431840967785</v>
+        <v>11.89370044882708</v>
       </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
@@ -2155,12 +2155,12 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>327.5028095393986</v>
+        <v>295.3629391829428</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>22.53846015202668</v>
+        <v>15.34660815434614</v>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr"/>
@@ -2181,12 +2181,12 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>294.0240022906991</v>
+        <v>280.7546698520774</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>16.04133371754528</v>
+        <v>13.64687074319993</v>
       </c>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>

</xml_diff>